<commit_message>
Document enrichment process and validate Task 1 outputs
</commit_message>
<xml_diff>
--- a/data/processed/ethiopia_fi_enriched.xlsx
+++ b/data/processed/ethiopia_fi_enriched.xlsx
@@ -607,11 +607,7 @@
       <c r="C2" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>high</t>
@@ -720,11 +716,7 @@
       <c r="C3" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>high</t>
@@ -829,11 +821,7 @@
       <c r="C4" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>high</t>
@@ -938,11 +926,7 @@
       <c r="C5" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>high</t>
@@ -1051,11 +1035,7 @@
       <c r="C6" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>high</t>
@@ -1164,11 +1144,7 @@
       <c r="C7" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>high</t>
@@ -1281,11 +1257,7 @@
       <c r="C8" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>high</t>
@@ -1390,11 +1362,7 @@
       <c r="C9" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>high</t>
@@ -1503,11 +1471,7 @@
       <c r="C10" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>high</t>
@@ -1618,11 +1582,7 @@
       <c r="C11" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>high</t>
@@ -1733,11 +1693,7 @@
       <c r="C12" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>high</t>
@@ -1846,11 +1802,7 @@
       <c r="C13" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>high</t>
@@ -1955,11 +1907,7 @@
       <c r="C14" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>high</t>
@@ -2060,11 +2008,7 @@
       <c r="C15" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>high</t>
@@ -2169,11 +2113,7 @@
       <c r="C16" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>high</t>
@@ -2288,11 +2228,7 @@
       <c r="C17" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>high</t>
@@ -2407,11 +2343,7 @@
       <c r="C18" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>high</t>
@@ -2526,11 +2458,7 @@
       <c r="C19" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>high</t>
@@ -2645,11 +2573,7 @@
       <c r="C20" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>high</t>
@@ -2760,11 +2684,7 @@
       <c r="C21" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>high</t>
@@ -2875,11 +2795,7 @@
       <c r="C22" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>high</t>
@@ -2990,11 +2906,7 @@
       <c r="C23" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>high</t>
@@ -3105,11 +3017,7 @@
       <c r="C24" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>high</t>
@@ -3210,11 +3118,7 @@
       <c r="C25" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>high</t>
@@ -3319,11 +3223,7 @@
       <c r="C26" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>high</t>
@@ -3428,11 +3328,7 @@
       <c r="C27" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>medium</t>
@@ -3541,11 +3437,7 @@
       <c r="C28" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>high</t>
@@ -3654,11 +3546,7 @@
       <c r="C29" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>medium</t>
@@ -3767,11 +3655,7 @@
       <c r="C30" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>high</t>
@@ -3880,11 +3764,7 @@
       <c r="C31" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>high</t>
@@ -3993,11 +3873,7 @@
       <c r="C32" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>high</t>
@@ -4106,11 +3982,7 @@
       <c r="C33" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>high</t>
@@ -4219,11 +4091,7 @@
       <c r="C34" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>medium</t>
@@ -4332,11 +4200,7 @@
       <c r="C35" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>high</t>
@@ -4439,11 +4303,7 @@
       <c r="C36" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>high</t>
@@ -4542,11 +4402,7 @@
       <c r="C37" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>high</t>
@@ -4645,11 +4501,7 @@
       <c r="C38" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>high</t>
@@ -4752,11 +4604,7 @@
       <c r="C39" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>high</t>
@@ -4855,11 +4703,7 @@
       <c r="C40" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>high</t>
@@ -4964,11 +4808,7 @@
       <c r="C41" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>high</t>
@@ -5069,11 +4909,7 @@
       <c r="C42" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>high</t>
@@ -5174,11 +5010,7 @@
       <c r="C43" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>high</t>
@@ -5285,11 +5117,7 @@
       <c r="C44" s="1" t="n">
         <v>45677</v>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Example_Trainee</t>
-        </is>
-      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>high</t>
@@ -7024,7 +6852,11 @@
       <c r="G59" t="n">
         <v>2011</v>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>

</xml_diff>